<commit_message>
Remove glitter eye makeup prompts
</commit_message>
<xml_diff>
--- a/data/prompt_pools.xlsx
+++ b/data/prompt_pools.xlsx
@@ -1390,7 +1390,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>宝石光猫眼妆，眼尾带银蓝细闪，冷白底妆像瓷面一样干净，眼尾黑色眼线明显上扬，浓密睫毛压出危险感，浅棕瞳孔带琥珀亮光，薄唇微反光，鼻梁高光锋利</t>
+          <t>冷艳猫眼妆，冷白底妆像瓷面一样干净，黑色眼线沿睫毛根部明显上扬，浓密睫毛压出危险感，浅棕瞳孔清透有神，薄唇只带轻微水光，鼻梁轮廓锋利</t>
         </is>
       </c>
     </row>
@@ -1427,7 +1427,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>夜色魅惑妆，眼尾带青紫细闪，底妆冷白且带轻微湿光，柔棕轻烟熏晕在眼尾，狐狸眼更狭长，睫毛浓密，原生薄唇覆透明无色唇彩只带轻微水光，脸颊泛出淡淡自然红润</t>
+          <t>夜色魅惑妆，底妆冷白且带轻微湿光，柔棕轻烟熏晕在眼尾，狐狸眼更狭长，眼周保持干净哑光，睫毛浓密，原生薄唇覆透明无色唇彩只带轻微水光，脸颊泛出淡淡自然红润</t>
         </is>
       </c>
     </row>
@@ -1464,7 +1464,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>高级私房妆，眼下带细小银色湿光，冷白底妆细腻无瑕，眼下有轻微粉色晕染，眼神湿润但更主动明亮，透明唇釉发亮，鼻梁侧影清楚，下巴下方有轻微阴影</t>
+          <t>高级私房妆，冷白底妆细腻无瑕，眼下只有轻微粉色柔雾晕染，眼神湿润但更主动明亮，透明唇釉发亮，鼻梁侧影清楚，下巴下方有轻微阴影</t>
         </is>
       </c>
     </row>
@@ -1501,7 +1501,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>舞台感亮片猫眼妆，银白细闪集中在眼头和眼尾，黑色眼线锐利，浅棕瞳孔带琥珀反光，原生薄唇微张直接</t>
+          <t>舞台感干净猫眼妆，眼头和眼尾保持清爽哑光，黑色眼线锐利，浅棕瞳孔清透，原生薄唇微张直接</t>
         </is>
       </c>
     </row>
@@ -1538,7 +1538,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>宝石光猫眼妆，眼尾带银蓝细闪，冷白底妆像瓷面一样细腻，黑色眼线锋利上挑，睫毛浓密压出侵略感，原生薄唇清亮水光，鼻梁高光锐利</t>
+          <t>冷艳猫眼妆，冷白底妆像瓷面一样细腻，黑色眼线锋利上挑，眼尾只用柔棕阴影拉长，睫毛浓密压出侵略感，原生薄唇清亮水光，鼻梁轮廓锐利</t>
         </is>
       </c>
     </row>
@@ -1575,7 +1575,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>湿润夜拍妆，眼尾带青灰反光，底妆冷白并带轻微潮湿光泽，眼尾轻烟熏向外拉长，浅棕瞳孔直勾勾反光，唇部是原生薄唇水光，脸颊微润</t>
+          <t>湿润夜拍妆，底妆冷白并带轻微潮湿光泽，眼尾轻烟熏向外拉长，眼周保持干净柔雾，浅棕瞳孔直视镜头，唇部是原生薄唇水光，脸颊微润</t>
         </is>
       </c>
     </row>
@@ -1612,7 +1612,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>舞台私房亮片妆，银蓝细闪集中在眼头和眼尾，黑色眼线强化狐狸眼，睫毛厚而卷翘，原生薄唇水光质地</t>
+          <t>舞台私房猫眼妆，眼头和眼尾保持干净哑光，黑色眼线强化狐狸眼，睫毛厚而卷翘，原生薄唇水光质地</t>
         </is>
       </c>
     </row>
@@ -1649,7 +1649,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>高压御姐妆，眼尾带香槟金细闪，底妆冷白无瑕，鼻梁侧影清楚，下巴下方有轻微阴影，眼尾深棕上扬，纤薄嘴唇保持原生湿亮，表情空间天然带强烈支配感</t>
+          <t>高压御姐妆，底妆冷白无瑕，鼻梁侧影清楚，下巴下方有轻微阴影，眼尾深棕上扬并保持柔雾质感，纤薄嘴唇保持原生湿亮，表情空间天然带强烈支配感</t>
         </is>
       </c>
     </row>
@@ -1686,7 +1686,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>暗调胶片妆，眼尾带暖金胶片反光，冷白底妆被暖光，压出柔和阴影，眼下带轻微自然红润，狐狸眼看起来沉重迷离，透明唇釉只，让薄唇边界轻微发亮，五官更有成人魅惑感</t>
+          <t>暗调胶片妆，冷白底妆被暖光压出柔和阴影，眼尾棕灰柔雾阴影拉长，眼下带轻微自然红润，狐狸眼看起来沉重迷离，透明唇釉只让薄唇边界轻微发亮，五官更有成人魅惑感</t>
         </is>
       </c>
     </row>
@@ -34574,7 +34574,7 @@
       </c>
       <c r="G856" t="inlineStr">
         <is>
-          <t>暗夜宝石光猫眼妆，眼尾带银蓝细闪，黑色眼线从内眼角拉到眼尾，睫毛浓密下压，眼下有淡淡自然红润，原生薄唇水光，脸部轮廓锋利而魅惑</t>
+          <t>暗夜冷艳猫眼妆，黑色眼线从内眼角拉到眼尾，眼尾保持干净柔雾，睫毛浓密下压，眼下有淡淡自然红润，原生薄唇水光，脸部轮廓锋利而魅惑</t>
         </is>
       </c>
     </row>

</xml_diff>